<commit_message>
Made logic of age parsing better
</commit_message>
<xml_diff>
--- a/output/voter_output.xlsx
+++ b/output/voter_output.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H890"/>
+  <dimension ref="A1:H891"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -672,7 +672,11 @@
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr"/>
-      <c r="G7" s="3" t="inlineStr"/>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -789,7 +793,11 @@
           <t>4</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr"/>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -901,7 +909,11 @@
           <t>4</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr"/>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -1549,7 +1561,11 @@
           <t>8</t>
         </is>
       </c>
-      <c r="G30" s="3" t="inlineStr"/>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -1585,7 +1601,11 @@
           <t>8</t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr"/>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -1661,7 +1681,11 @@
           <t>8</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr"/>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -1697,7 +1721,11 @@
           <t>8A</t>
         </is>
       </c>
-      <c r="G34" s="3" t="inlineStr"/>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -2281,7 +2309,11 @@
           <t>11</t>
         </is>
       </c>
-      <c r="G49" s="3" t="inlineStr"/>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -2505,7 +2537,11 @@
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr"/>
-      <c r="G55" s="3" t="inlineStr"/>
+      <c r="G55" s="3" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
       <c r="H55" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -2861,7 +2897,11 @@
           <t>16</t>
         </is>
       </c>
-      <c r="G64" s="3" t="inlineStr"/>
+      <c r="G64" s="3" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
       <c r="H64" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -3165,7 +3205,11 @@
           <t>17</t>
         </is>
       </c>
-      <c r="G72" s="3" t="inlineStr"/>
+      <c r="G72" s="3" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
       <c r="H72" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -3197,7 +3241,11 @@
         </is>
       </c>
       <c r="F73" s="3" t="inlineStr"/>
-      <c r="G73" s="3" t="inlineStr"/>
+      <c r="G73" s="3" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
       <c r="H73" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -3313,7 +3361,11 @@
           <t>17</t>
         </is>
       </c>
-      <c r="G76" s="3" t="inlineStr"/>
+      <c r="G76" s="3" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
       <c r="H76" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -3645,7 +3697,11 @@
           <t>18</t>
         </is>
       </c>
-      <c r="G85" s="3" t="inlineStr"/>
+      <c r="G85" s="3" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
       <c r="H85" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -3877,7 +3933,11 @@
           <t>19</t>
         </is>
       </c>
-      <c r="G91" s="3" t="inlineStr"/>
+      <c r="G91" s="3" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
       <c r="H91" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -3953,7 +4013,11 @@
           <t>194</t>
         </is>
       </c>
-      <c r="G93" s="3" t="inlineStr"/>
+      <c r="G93" s="3" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
       <c r="H93" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -3989,7 +4053,11 @@
           <t>194</t>
         </is>
       </c>
-      <c r="G94" s="3" t="inlineStr"/>
+      <c r="G94" s="3" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
       <c r="H94" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -4265,7 +4333,11 @@
           <t>21</t>
         </is>
       </c>
-      <c r="G101" s="3" t="inlineStr"/>
+      <c r="G101" s="3" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
       <c r="H101" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -4801,7 +4873,11 @@
         </is>
       </c>
       <c r="F115" s="3" t="inlineStr"/>
-      <c r="G115" s="3" t="inlineStr"/>
+      <c r="G115" s="3" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
       <c r="H115" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -4989,7 +5065,11 @@
           <t>24</t>
         </is>
       </c>
-      <c r="G120" s="3" t="inlineStr"/>
+      <c r="G120" s="3" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
       <c r="H120" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -5497,7 +5577,11 @@
           <t>45</t>
         </is>
       </c>
-      <c r="G133" s="3" t="inlineStr"/>
+      <c r="G133" s="3" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
       <c r="H133" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -5613,7 +5697,11 @@
           <t>No:2,Gayathri Homes,3rd</t>
         </is>
       </c>
-      <c r="G136" s="3" t="inlineStr"/>
+      <c r="G136" s="3" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
       <c r="H136" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -5845,7 +5933,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="G142" s="3" t="inlineStr"/>
+      <c r="G142" s="3" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
       <c r="H142" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -6229,7 +6321,11 @@
         </is>
       </c>
       <c r="F152" s="3" t="inlineStr"/>
-      <c r="G152" s="3" t="inlineStr"/>
+      <c r="G152" s="3" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
       <c r="H152" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -6689,7 +6785,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="G164" s="3" t="inlineStr"/>
+      <c r="G164" s="3" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
       <c r="H164" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -6845,7 +6945,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="G168" s="3" t="inlineStr"/>
+      <c r="G168" s="3" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="H168" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -6881,7 +6985,11 @@
           <t>1A</t>
         </is>
       </c>
-      <c r="G169" s="3" t="inlineStr"/>
+      <c r="G169" s="3" t="inlineStr">
+        <is>
+          <t>95</t>
+        </is>
+      </c>
       <c r="H169" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -6917,7 +7025,11 @@
           <t>1A</t>
         </is>
       </c>
-      <c r="G170" s="3" t="inlineStr"/>
+      <c r="G170" s="3" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
       <c r="H170" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -7033,7 +7145,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="G173" s="3" t="inlineStr"/>
+      <c r="G173" s="3" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
       <c r="H173" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -7373,7 +7489,11 @@
         </is>
       </c>
       <c r="F182" s="3" t="inlineStr"/>
-      <c r="G182" s="3" t="inlineStr"/>
+      <c r="G182" s="3" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
       <c r="H182" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -8025,7 +8145,11 @@
           <t>4</t>
         </is>
       </c>
-      <c r="G199" s="3" t="inlineStr"/>
+      <c r="G199" s="3" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
       <c r="H199" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -8061,7 +8185,11 @@
           <t>5</t>
         </is>
       </c>
-      <c r="G200" s="3" t="inlineStr"/>
+      <c r="G200" s="3" t="inlineStr">
+        <is>
+          <t>83</t>
+        </is>
+      </c>
       <c r="H200" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -8177,7 +8305,11 @@
           <t>5</t>
         </is>
       </c>
-      <c r="G203" s="3" t="inlineStr"/>
+      <c r="G203" s="3" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
       <c r="H203" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -8514,7 +8646,11 @@
         </is>
       </c>
       <c r="F212" s="3" t="inlineStr"/>
-      <c r="G212" s="3" t="inlineStr"/>
+      <c r="G212" s="3" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
       <c r="H212" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -8704,7 +8840,7 @@
       </c>
       <c r="G217" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>27</t>
         </is>
       </c>
       <c r="H217" s="3" t="inlineStr">
@@ -8962,7 +9098,11 @@
         </is>
       </c>
       <c r="F224" s="3" t="inlineStr"/>
-      <c r="G224" s="3" t="inlineStr"/>
+      <c r="G224" s="3" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
       <c r="H224" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -9158,7 +9298,11 @@
           <t>7</t>
         </is>
       </c>
-      <c r="G229" s="3" t="inlineStr"/>
+      <c r="G229" s="3" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
       <c r="H229" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -9194,7 +9338,11 @@
           <t>7</t>
         </is>
       </c>
-      <c r="G230" s="3" t="inlineStr"/>
+      <c r="G230" s="3" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
       <c r="H230" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -9310,7 +9458,11 @@
           <t>7A 8A</t>
         </is>
       </c>
-      <c r="G233" s="3" t="inlineStr"/>
+      <c r="G233" s="3" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
       <c r="H233" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -9346,7 +9498,11 @@
           <t>7A 8A</t>
         </is>
       </c>
-      <c r="G234" s="3" t="inlineStr"/>
+      <c r="G234" s="3" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
       <c r="H234" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -9538,7 +9694,11 @@
           <t>8</t>
         </is>
       </c>
-      <c r="G239" s="3" t="inlineStr"/>
+      <c r="G239" s="3" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
       <c r="H239" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -9646,7 +9806,11 @@
         </is>
       </c>
       <c r="F242" s="3" t="inlineStr"/>
-      <c r="G242" s="3" t="inlineStr"/>
+      <c r="G242" s="3" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
       <c r="H242" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -9754,7 +9918,11 @@
           <t>9</t>
         </is>
       </c>
-      <c r="G245" s="3" t="inlineStr"/>
+      <c r="G245" s="3" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
       <c r="H245" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -10226,7 +10394,11 @@
         </is>
       </c>
       <c r="F257" s="3" t="inlineStr"/>
-      <c r="G257" s="3" t="inlineStr"/>
+      <c r="G257" s="3" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
       <c r="H257" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -10262,7 +10434,11 @@
           <t>11</t>
         </is>
       </c>
-      <c r="G258" s="3" t="inlineStr"/>
+      <c r="G258" s="3" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
       <c r="H258" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -10298,7 +10474,11 @@
           <t>11</t>
         </is>
       </c>
-      <c r="G259" s="3" t="inlineStr"/>
+      <c r="G259" s="3" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
       <c r="H259" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -10414,7 +10594,11 @@
           <t>11</t>
         </is>
       </c>
-      <c r="G262" s="3" t="inlineStr"/>
+      <c r="G262" s="3" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
       <c r="H262" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -10806,7 +10990,11 @@
           <t>12</t>
         </is>
       </c>
-      <c r="G272" s="3" t="inlineStr"/>
+      <c r="G272" s="3" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
       <c r="H272" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -11034,7 +11222,11 @@
           <t>12</t>
         </is>
       </c>
-      <c r="G278" s="3" t="inlineStr"/>
+      <c r="G278" s="3" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
       <c r="H278" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -11490,7 +11682,11 @@
           <t>13</t>
         </is>
       </c>
-      <c r="G290" s="3" t="inlineStr"/>
+      <c r="G290" s="3" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
       <c r="H290" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -11838,7 +12034,11 @@
           <t>14B</t>
         </is>
       </c>
-      <c r="G299" s="3" t="inlineStr"/>
+      <c r="G299" s="3" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
       <c r="H299" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -12186,7 +12386,11 @@
           <t>15</t>
         </is>
       </c>
-      <c r="G308" s="3" t="inlineStr"/>
+      <c r="G308" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
       <c r="H308" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -12342,7 +12546,11 @@
           <t>15</t>
         </is>
       </c>
-      <c r="G312" s="3" t="inlineStr"/>
+      <c r="G312" s="3" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
       <c r="H312" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -12650,7 +12858,11 @@
           <t>15.</t>
         </is>
       </c>
-      <c r="G320" s="3" t="inlineStr"/>
+      <c r="G320" s="3" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
       <c r="H320" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -12726,7 +12938,11 @@
           <t>15</t>
         </is>
       </c>
-      <c r="G322" s="3" t="inlineStr"/>
+      <c r="G322" s="3" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
       <c r="H322" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -12762,7 +12978,11 @@
           <t>15</t>
         </is>
       </c>
-      <c r="G323" s="3" t="inlineStr"/>
+      <c r="G323" s="3" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
       <c r="H323" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -13154,7 +13374,11 @@
           <t>15B</t>
         </is>
       </c>
-      <c r="G333" s="3" t="inlineStr"/>
+      <c r="G333" s="3" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
       <c r="H333" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -13386,7 +13610,11 @@
           <t>16</t>
         </is>
       </c>
-      <c r="G339" s="3" t="inlineStr"/>
+      <c r="G339" s="3" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
       <c r="H339" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -13926,7 +14154,11 @@
           <t>17</t>
         </is>
       </c>
-      <c r="G353" s="3" t="inlineStr"/>
+      <c r="G353" s="3" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
+      </c>
       <c r="H353" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -14162,7 +14394,11 @@
           <t>17</t>
         </is>
       </c>
-      <c r="G359" s="3" t="inlineStr"/>
+      <c r="G359" s="3" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
       <c r="H359" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -14754,7 +14990,11 @@
         </is>
       </c>
       <c r="F374" s="3" t="inlineStr"/>
-      <c r="G374" s="3" t="inlineStr"/>
+      <c r="G374" s="3" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
       <c r="H374" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -14982,7 +15222,11 @@
           <t>20</t>
         </is>
       </c>
-      <c r="G380" s="3" t="inlineStr"/>
+      <c r="G380" s="3" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
       <c r="H380" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -15054,7 +15298,11 @@
           <t>20</t>
         </is>
       </c>
-      <c r="G382" s="3" t="inlineStr"/>
+      <c r="G382" s="3" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
       <c r="H382" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -15090,7 +15338,11 @@
           <t>20</t>
         </is>
       </c>
-      <c r="G383" s="3" t="inlineStr"/>
+      <c r="G383" s="3" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
       <c r="H383" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -15206,7 +15458,11 @@
           <t>20B.</t>
         </is>
       </c>
-      <c r="G386" s="3" t="inlineStr"/>
+      <c r="G386" s="3" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
       <c r="H386" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -16058,7 +16314,11 @@
           <t>23</t>
         </is>
       </c>
-      <c r="G408" s="3" t="inlineStr"/>
+      <c r="G408" s="3" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
       <c r="H408" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -16366,7 +16626,11 @@
           <t>23</t>
         </is>
       </c>
-      <c r="G416" s="3" t="inlineStr"/>
+      <c r="G416" s="3" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
       <c r="H416" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -16598,7 +16862,11 @@
         </is>
       </c>
       <c r="F422" s="3" t="inlineStr"/>
-      <c r="G422" s="3" t="inlineStr"/>
+      <c r="G422" s="3" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
       <c r="H422" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -16834,7 +17102,11 @@
           <t>25</t>
         </is>
       </c>
-      <c r="G428" s="3" t="inlineStr"/>
+      <c r="G428" s="3" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
       <c r="H428" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -16942,7 +17214,11 @@
           <t>25,</t>
         </is>
       </c>
-      <c r="G431" s="3" t="inlineStr"/>
+      <c r="G431" s="3" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
       <c r="H431" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -17242,7 +17518,11 @@
           <t>27</t>
         </is>
       </c>
-      <c r="G439" s="3" t="inlineStr"/>
+      <c r="G439" s="3" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
       <c r="H439" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -17278,7 +17558,11 @@
           <t>27</t>
         </is>
       </c>
-      <c r="G440" s="3" t="inlineStr"/>
+      <c r="G440" s="3" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
       <c r="H440" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -17354,7 +17638,11 @@
           <t>27</t>
         </is>
       </c>
-      <c r="G442" s="3" t="inlineStr"/>
+      <c r="G442" s="3" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
       <c r="H442" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -17390,7 +17678,11 @@
           <t>27</t>
         </is>
       </c>
-      <c r="G443" s="3" t="inlineStr"/>
+      <c r="G443" s="3" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
       <c r="H443" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -17974,7 +18266,11 @@
         </is>
       </c>
       <c r="F458" s="3" t="inlineStr"/>
-      <c r="G458" s="3" t="inlineStr"/>
+      <c r="G458" s="3" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
       <c r="H458" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -18210,7 +18506,11 @@
           <t>30</t>
         </is>
       </c>
-      <c r="G464" s="3" t="inlineStr"/>
+      <c r="G464" s="3" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
       <c r="H464" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -18318,7 +18618,11 @@
           <t>31</t>
         </is>
       </c>
-      <c r="G467" s="3" t="inlineStr"/>
+      <c r="G467" s="3" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
       <c r="H467" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -18354,7 +18658,11 @@
           <t>31</t>
         </is>
       </c>
-      <c r="G468" s="3" t="inlineStr"/>
+      <c r="G468" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
       <c r="H468" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -18510,7 +18818,11 @@
           <t>31</t>
         </is>
       </c>
-      <c r="G472" s="3" t="inlineStr"/>
+      <c r="G472" s="3" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
       <c r="H472" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -18546,7 +18858,11 @@
           <t>31</t>
         </is>
       </c>
-      <c r="G473" s="3" t="inlineStr"/>
+      <c r="G473" s="3" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
       <c r="H473" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -18890,7 +19206,11 @@
           <t>32</t>
         </is>
       </c>
-      <c r="G482" s="3" t="inlineStr"/>
+      <c r="G482" s="3" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
       <c r="H482" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -18926,7 +19246,11 @@
           <t>33</t>
         </is>
       </c>
-      <c r="G483" s="3" t="inlineStr"/>
+      <c r="G483" s="3" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
       <c r="H483" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -19118,7 +19442,11 @@
         </is>
       </c>
       <c r="F488" s="3" t="inlineStr"/>
-      <c r="G488" s="3" t="inlineStr"/>
+      <c r="G488" s="3" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
       <c r="H488" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -19346,7 +19674,11 @@
         </is>
       </c>
       <c r="F494" s="3" t="inlineStr"/>
-      <c r="G494" s="3" t="inlineStr"/>
+      <c r="G494" s="3" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
       <c r="H494" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -19582,7 +19914,11 @@
           <t>34</t>
         </is>
       </c>
-      <c r="G500" s="3" t="inlineStr"/>
+      <c r="G500" s="3" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
       <c r="H500" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -19658,7 +19994,11 @@
           <t>34</t>
         </is>
       </c>
-      <c r="G502" s="3" t="inlineStr"/>
+      <c r="G502" s="3" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
       <c r="H502" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -19694,7 +20034,11 @@
           <t>34</t>
         </is>
       </c>
-      <c r="G503" s="3" t="inlineStr"/>
+      <c r="G503" s="3" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
       <c r="H503" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -20628,7 +20972,11 @@
           <t>36</t>
         </is>
       </c>
-      <c r="G527" s="3" t="inlineStr"/>
+      <c r="G527" s="3" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
       <c r="H527" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -20704,7 +21052,11 @@
           <t>36</t>
         </is>
       </c>
-      <c r="G529" s="3" t="inlineStr"/>
+      <c r="G529" s="3" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
       <c r="H529" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -20740,7 +21092,11 @@
           <t>36/52</t>
         </is>
       </c>
-      <c r="G530" s="3" t="inlineStr"/>
+      <c r="G530" s="3" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
       <c r="H530" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -20852,7 +21208,11 @@
           <t>37</t>
         </is>
       </c>
-      <c r="G533" s="3" t="inlineStr"/>
+      <c r="G533" s="3" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
       <c r="H533" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -21200,7 +21560,11 @@
           <t>38</t>
         </is>
       </c>
-      <c r="G542" s="3" t="inlineStr"/>
+      <c r="G542" s="3" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
       <c r="H542" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -21660,7 +22024,11 @@
           <t>39B.</t>
         </is>
       </c>
-      <c r="G554" s="3" t="inlineStr"/>
+      <c r="G554" s="3" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
       <c r="H554" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -21816,7 +22184,11 @@
           <t>40</t>
         </is>
       </c>
-      <c r="G558" s="3" t="inlineStr"/>
+      <c r="G558" s="3" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
       <c r="H558" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -21892,7 +22264,11 @@
           <t>41</t>
         </is>
       </c>
-      <c r="G560" s="3" t="inlineStr"/>
+      <c r="G560" s="3" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
       <c r="H560" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -22004,7 +22380,11 @@
           <t>41</t>
         </is>
       </c>
-      <c r="G563" s="3" t="inlineStr"/>
+      <c r="G563" s="3" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
       <c r="H563" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -22353,7 +22733,11 @@
           <t>41</t>
         </is>
       </c>
-      <c r="G572" s="3" t="inlineStr"/>
+      <c r="G572" s="3" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
       <c r="H572" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -22381,7 +22765,11 @@
           <t>42</t>
         </is>
       </c>
-      <c r="G573" s="3" t="inlineStr"/>
+      <c r="G573" s="3" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
       <c r="H573" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -22805,7 +23193,11 @@
           <t>44</t>
         </is>
       </c>
-      <c r="G584" s="3" t="inlineStr"/>
+      <c r="G584" s="3" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
       <c r="H584" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -23001,7 +23393,11 @@
           <t>45</t>
         </is>
       </c>
-      <c r="G589" s="3" t="inlineStr"/>
+      <c r="G589" s="3" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
       <c r="H589" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -23157,7 +23553,11 @@
           <t>46</t>
         </is>
       </c>
-      <c r="G593" s="3" t="inlineStr"/>
+      <c r="G593" s="3" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
       <c r="H593" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -23633,7 +24033,11 @@
           <t>48</t>
         </is>
       </c>
-      <c r="G605" s="3" t="inlineStr"/>
+      <c r="G605" s="3" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
       <c r="H605" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -23789,7 +24193,11 @@
           <t>48</t>
         </is>
       </c>
-      <c r="G609" s="3" t="inlineStr"/>
+      <c r="G609" s="3" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
       <c r="H609" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -23897,7 +24305,11 @@
           <t>49</t>
         </is>
       </c>
-      <c r="G612" s="3" t="inlineStr"/>
+      <c r="G612" s="3" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
       <c r="H612" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -24053,7 +24465,11 @@
           <t>49</t>
         </is>
       </c>
-      <c r="G616" s="3" t="inlineStr"/>
+      <c r="G616" s="3" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
       <c r="H616" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -24129,7 +24545,11 @@
           <t>50</t>
         </is>
       </c>
-      <c r="G618" s="3" t="inlineStr"/>
+      <c r="G618" s="3" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
       <c r="H618" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -24205,7 +24625,11 @@
           <t>51</t>
         </is>
       </c>
-      <c r="G620" s="3" t="inlineStr"/>
+      <c r="G620" s="3" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
       <c r="H620" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -24321,7 +24745,11 @@
           <t>51</t>
         </is>
       </c>
-      <c r="G623" s="3" t="inlineStr"/>
+      <c r="G623" s="3" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
       <c r="H623" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -25293,7 +25721,11 @@
           <t>59</t>
         </is>
       </c>
-      <c r="G648" s="3" t="inlineStr"/>
+      <c r="G648" s="3" t="inlineStr">
+        <is>
+          <t>71</t>
+        </is>
+      </c>
       <c r="H648" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -25329,7 +25761,11 @@
           <t>59</t>
         </is>
       </c>
-      <c r="G649" s="3" t="inlineStr"/>
+      <c r="G649" s="3" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
       <c r="H649" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -25365,7 +25801,11 @@
           <t>59</t>
         </is>
       </c>
-      <c r="G650" s="3" t="inlineStr"/>
+      <c r="G650" s="3" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
       <c r="H650" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -25481,7 +25921,11 @@
           <t>61</t>
         </is>
       </c>
-      <c r="G653" s="3" t="inlineStr"/>
+      <c r="G653" s="3" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
       <c r="H653" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -26289,7 +26733,11 @@
         </is>
       </c>
       <c r="F674" s="3" t="inlineStr"/>
-      <c r="G674" s="3" t="inlineStr"/>
+      <c r="G674" s="3" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
       <c r="H674" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -26365,7 +26813,11 @@
           <t>65</t>
         </is>
       </c>
-      <c r="G676" s="3" t="inlineStr"/>
+      <c r="G676" s="3" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
       <c r="H676" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -26481,7 +26933,11 @@
           <t>65</t>
         </is>
       </c>
-      <c r="G679" s="3" t="inlineStr"/>
+      <c r="G679" s="3" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
       <c r="H679" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -26589,7 +27045,11 @@
           <t>65,</t>
         </is>
       </c>
-      <c r="G682" s="3" t="inlineStr"/>
+      <c r="G682" s="3" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
       <c r="H682" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -26625,7 +27085,11 @@
           <t>65</t>
         </is>
       </c>
-      <c r="G683" s="3" t="inlineStr"/>
+      <c r="G683" s="3" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
       <c r="H683" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -26977,7 +27441,11 @@
         </is>
       </c>
       <c r="F692" s="3" t="inlineStr"/>
-      <c r="G692" s="3" t="inlineStr"/>
+      <c r="G692" s="3" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
       <c r="H692" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -27013,7 +27481,11 @@
           <t>71</t>
         </is>
       </c>
-      <c r="G693" s="3" t="inlineStr"/>
+      <c r="G693" s="3" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
       <c r="H693" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -27353,7 +27825,11 @@
           <t>77</t>
         </is>
       </c>
-      <c r="G702" s="3" t="inlineStr"/>
+      <c r="G702" s="3" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
       <c r="H702" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -27621,7 +28097,11 @@
           <t>77</t>
         </is>
       </c>
-      <c r="G709" s="3" t="inlineStr"/>
+      <c r="G709" s="3" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
       <c r="H709" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -27737,7 +28217,11 @@
           <t>77</t>
         </is>
       </c>
-      <c r="G712" s="3" t="inlineStr"/>
+      <c r="G712" s="3" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
       <c r="H712" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -27773,7 +28257,11 @@
           <t>77</t>
         </is>
       </c>
-      <c r="G713" s="3" t="inlineStr"/>
+      <c r="G713" s="3" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
       <c r="H713" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -27889,7 +28377,11 @@
           <t>77</t>
         </is>
       </c>
-      <c r="G716" s="3" t="inlineStr"/>
+      <c r="G716" s="3" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
       <c r="H716" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -28125,7 +28617,11 @@
           <t>78</t>
         </is>
       </c>
-      <c r="G722" s="3" t="inlineStr"/>
+      <c r="G722" s="3" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
       <c r="H722" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -28161,7 +28657,11 @@
           <t>78</t>
         </is>
       </c>
-      <c r="G723" s="3" t="inlineStr"/>
+      <c r="G723" s="3" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
       <c r="H723" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -28709,7 +29209,11 @@
           <t>60</t>
         </is>
       </c>
-      <c r="G737" s="3" t="inlineStr"/>
+      <c r="G737" s="3" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
       <c r="H737" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -28825,7 +29329,11 @@
           <t>80</t>
         </is>
       </c>
-      <c r="G740" s="3" t="inlineStr"/>
+      <c r="G740" s="3" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
       <c r="H740" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -29221,7 +29729,11 @@
           <t>81</t>
         </is>
       </c>
-      <c r="G750" s="3" t="inlineStr"/>
+      <c r="G750" s="3" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
       <c r="H750" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -29337,7 +29849,11 @@
           <t>81</t>
         </is>
       </c>
-      <c r="G753" s="3" t="inlineStr"/>
+      <c r="G753" s="3" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
       <c r="H753" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -29573,7 +30089,11 @@
           <t>82</t>
         </is>
       </c>
-      <c r="G759" s="3" t="inlineStr"/>
+      <c r="G759" s="3" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
       <c r="H759" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -29949,7 +30469,11 @@
           <t>83</t>
         </is>
       </c>
-      <c r="G769" s="3" t="inlineStr"/>
+      <c r="G769" s="3" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
       <c r="H769" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -29985,7 +30509,11 @@
           <t>83</t>
         </is>
       </c>
-      <c r="G770" s="3" t="inlineStr"/>
+      <c r="G770" s="3" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
       <c r="H770" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -30061,7 +30589,11 @@
           <t>83</t>
         </is>
       </c>
-      <c r="G772" s="3" t="inlineStr"/>
+      <c r="G772" s="3" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
       <c r="H772" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -30937,7 +31469,11 @@
           <t>85</t>
         </is>
       </c>
-      <c r="G794" s="3" t="inlineStr"/>
+      <c r="G794" s="3" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
       <c r="H794" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -31005,7 +31541,11 @@
           <t>85</t>
         </is>
       </c>
-      <c r="G796" s="3" t="inlineStr"/>
+      <c r="G796" s="3" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
       <c r="H796" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -31281,7 +31821,11 @@
           <t>87</t>
         </is>
       </c>
-      <c r="G803" s="3" t="inlineStr"/>
+      <c r="G803" s="3" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
       <c r="H803" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -31869,7 +32413,11 @@
           <t>95</t>
         </is>
       </c>
-      <c r="G818" s="3" t="inlineStr"/>
+      <c r="G818" s="3" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
       <c r="H818" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -32098,7 +32646,11 @@
           <t>100</t>
         </is>
       </c>
-      <c r="G824" s="3" t="inlineStr"/>
+      <c r="G824" s="3" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
       <c r="H824" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -32326,7 +32878,11 @@
           <t>103</t>
         </is>
       </c>
-      <c r="G830" s="3" t="inlineStr"/>
+      <c r="G830" s="3" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
       <c r="H830" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -32402,7 +32958,11 @@
           <t>103</t>
         </is>
       </c>
-      <c r="G832" s="3" t="inlineStr"/>
+      <c r="G832" s="3" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
       <c r="H832" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -32438,7 +32998,11 @@
           <t>103</t>
         </is>
       </c>
-      <c r="G833" s="3" t="inlineStr"/>
+      <c r="G833" s="3" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
       <c r="H833" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -32791,7 +33355,11 @@
           <t>107</t>
         </is>
       </c>
-      <c r="G842" s="3" t="inlineStr"/>
+      <c r="G842" s="3" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
       <c r="H842" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -32907,7 +33475,11 @@
           <t>110</t>
         </is>
       </c>
-      <c r="G845" s="3" t="inlineStr"/>
+      <c r="G845" s="3" t="inlineStr">
+        <is>
+          <t>95</t>
+        </is>
+      </c>
       <c r="H845" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -33255,7 +33827,11 @@
           <t>111</t>
         </is>
       </c>
-      <c r="G854" s="3" t="inlineStr"/>
+      <c r="G854" s="3" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
       <c r="H854" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -33447,7 +34023,11 @@
           <t>113</t>
         </is>
       </c>
-      <c r="G859" s="3" t="inlineStr"/>
+      <c r="G859" s="3" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
       <c r="H859" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -33479,7 +34059,11 @@
           <t>113</t>
         </is>
       </c>
-      <c r="G860" s="3" t="inlineStr"/>
+      <c r="G860" s="3" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
       <c r="H860" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -33555,7 +34139,11 @@
           <t>116</t>
         </is>
       </c>
-      <c r="G862" s="3" t="inlineStr"/>
+      <c r="G862" s="3" t="inlineStr">
+        <is>
+          <t>82</t>
+        </is>
+      </c>
       <c r="H862" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -33591,7 +34179,11 @@
           <t>116</t>
         </is>
       </c>
-      <c r="G863" s="3" t="inlineStr"/>
+      <c r="G863" s="3" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
       <c r="H863" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -33943,7 +34535,11 @@
         </is>
       </c>
       <c r="F872" s="3" t="inlineStr"/>
-      <c r="G872" s="3" t="inlineStr"/>
+      <c r="G872" s="3" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
       <c r="H872" s="3" t="inlineStr">
         <is>
           <t>Female</t>
@@ -34603,7 +35199,11 @@
           <t>Plot 33 4th cross</t>
         </is>
       </c>
-      <c r="G889" s="3" t="inlineStr"/>
+      <c r="G889" s="3" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
       <c r="H889" s="3" t="inlineStr">
         <is>
           <t>Male</t>
@@ -34643,6 +35243,46 @@
       <c r="H890" s="3" t="inlineStr">
         <is>
           <t>Female</t>
+        </is>
+      </c>
+    </row>
+    <row r="891">
+      <c r="A891" s="3" t="n">
+        <v>889</v>
+      </c>
+      <c r="B891" s="3" t="inlineStr">
+        <is>
+          <t>IPD0229732</t>
+        </is>
+      </c>
+      <c r="C891" s="3" t="inlineStr">
+        <is>
+          <t>KAMALUDIN</t>
+        </is>
+      </c>
+      <c r="D891" s="3" t="inlineStr">
+        <is>
+          <t>MOHAMMED CHERIEF</t>
+        </is>
+      </c>
+      <c r="E891" s="3" t="inlineStr">
+        <is>
+          <t>Father</t>
+        </is>
+      </c>
+      <c r="F891" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G891" s="3" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="H891" s="3" t="inlineStr">
+        <is>
+          <t>Male</t>
         </is>
       </c>
     </row>

</xml_diff>